<commit_message>
Added login data parametrization and admin page methods
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/Login.xlsx
+++ b/src/test/resources/TestData/Login.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\seleniumautomationown\adminorangeHRMSelenium\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB571D81-11DA-4B84-A71E-BF727FCC6439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F458DA28-93EC-4FD1-AA17-22D6353ED75A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{67A203F3-3266-43CB-8019-A7CC6E553D1A}"/>
   </bookViews>
   <sheets>
-    <sheet name="verifyValidLogin" sheetId="1" r:id="rId1"/>
-    <sheet name="verifyInValidLogin" sheetId="2" r:id="rId2"/>
+    <sheet name="verifyLogin" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="7">
   <si>
     <t>username</t>
   </si>
@@ -51,10 +50,13 @@
     <t>admin123</t>
   </si>
   <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>test123</t>
+    <t>expectedResult</t>
+  </si>
+  <si>
+    <t>Success</t>
+  </si>
+  <si>
+    <t>Requried</t>
   </si>
 </sst>
 </file>
@@ -426,49 +428,50 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{142A7EA3-548A-4207-9529-B0A866FA3860}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.6640625" customWidth="1"/>
+    <col min="2" max="2" width="11.5546875" customWidth="1"/>
+    <col min="3" max="3" width="18.77734375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B995FE42-E797-4DC6-BA0A-CA3BF2BE6B08}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>